<commit_message>
fix: harden MCP eval infrastructure and benchmark cases
</commit_message>
<xml_diff>
--- a/tasks/finalpool/canvas-announcement-summary/groundtruth_workspace/Course_Announcements.xlsx
+++ b/tasks/finalpool/canvas-announcement-summary/groundtruth_workspace/Course_Announcements.xlsx
@@ -450,12 +450,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025-09-05 01:12:34.377828+02:00</t>
+          <t>2025-09-04</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-03-07 03:00:00+01:00</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
@@ -470,12 +470,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025-09-12 01:12:34.377828+02:00</t>
+          <t>2025-09-11</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-05 00:12:34.377828+01:00</t>
+          <t>2026-03-04</t>
         </is>
       </c>
     </row>
@@ -490,12 +490,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025-09-26 01:12:34.377828+02:00</t>
+          <t>2025-09-25</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-16 00:12:34.377828+01:00</t>
+          <t>2026-02-15</t>
         </is>
       </c>
     </row>
@@ -510,12 +510,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2025-09-26 01:12:34.377828+02:00</t>
+          <t>2025-09-25</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-14 00:12:34.377828+01:00</t>
+          <t>2026-02-13</t>
         </is>
       </c>
     </row>
@@ -530,12 +530,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2025-08-20 01:12:34.377828+02:00</t>
+          <t>2025-08-19</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-02-07 00:12:34.377828+01:00</t>
+          <t>2026-02-06</t>
         </is>
       </c>
     </row>
@@ -550,12 +550,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2025-08-18 01:12:34.377828+02:00</t>
+          <t>2025-08-17</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-02-08 00:12:34.377828+01:00</t>
+          <t>2026-02-07</t>
         </is>
       </c>
     </row>
@@ -570,12 +570,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025-09-21 01:12:34.377828+02:00</t>
+          <t>2025-09-20</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-02-15 00:12:34.377828+01:00</t>
+          <t>2026-02-14</t>
         </is>
       </c>
     </row>
@@ -590,12 +590,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2025-10-14 01:12:34.377828+02:00</t>
+          <t>2025-10-13</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2025-11-08 00:12:34.377828+01:00</t>
+          <t>2025-11-07</t>
         </is>
       </c>
     </row>
@@ -610,12 +610,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2025-08-24 01:12:34.377828+02:00</t>
+          <t>2025-08-23</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-02-14 00:12:34.377828+01:00</t>
+          <t>2026-02-13</t>
         </is>
       </c>
     </row>
@@ -630,12 +630,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2025-08-26 01:12:34.377828+02:00</t>
+          <t>2025-08-25</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-02-25 00:12:34.377828+01:00</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -650,12 +650,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2025-09-24 01:12:34.377828+02:00</t>
+          <t>2025-09-23</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-02-19 00:12:34.377828+01:00</t>
+          <t>2026-02-18</t>
         </is>
       </c>
     </row>
@@ -670,12 +670,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2025-09-03 01:12:34.377828+02:00</t>
+          <t>2025-09-02</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2025-12-29 00:12:34.377828+01:00</t>
+          <t>2025-12-28</t>
         </is>
       </c>
     </row>
@@ -690,12 +690,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2025-08-24 01:12:34.377828+02:00</t>
+          <t>2025-08-23</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-01-31 00:12:34.377828+01:00</t>
+          <t>2026-01-30</t>
         </is>
       </c>
     </row>
@@ -710,12 +710,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2025-11-18 00:12:34.377828+01:00</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-02-20 00:12:34.377828+01:00</t>
+          <t>2026-02-19</t>
         </is>
       </c>
     </row>
@@ -730,12 +730,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2025-09-13 01:12:34.377828+02:00</t>
+          <t>2025-09-12</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-01-28 00:12:34.377828+01:00</t>
+          <t>2026-01-27</t>
         </is>
       </c>
     </row>
@@ -750,12 +750,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2025-09-20 01:12:34.377828+02:00</t>
+          <t>2025-09-19</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-02-22 00:12:34.377828+01:00</t>
+          <t>2026-02-21</t>
         </is>
       </c>
     </row>
@@ -770,12 +770,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2025-09-02 01:12:34.377828+02:00</t>
+          <t>2025-09-01</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2025-12-17 00:12:34.377828+01:00</t>
+          <t>2025-12-16</t>
         </is>
       </c>
     </row>
@@ -790,12 +790,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2025-09-28 01:12:34.377828+02:00</t>
+          <t>2025-09-27</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2025-12-14 00:12:34.377828+01:00</t>
+          <t>2025-12-13</t>
         </is>
       </c>
     </row>
@@ -810,12 +810,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2025-09-01 01:12:34.377828+02:00</t>
+          <t>2025-08-31</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2025-12-03 00:12:34.377828+01:00</t>
+          <t>2025-12-02</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2025-11-21 00:12:34.377828+01:00</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-02-18 00:12:34.377828+01:00</t>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>
@@ -850,12 +850,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2025-11-16 00:12:34.377828+01:00</t>
+          <t>2025-11-15</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-01-26 00:12:34.377828+01:00</t>
+          <t>2026-01-25</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2025-10-11 01:12:34.377828+02:00</t>
+          <t>2025-10-10</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2025-12-23 00:12:34.377828+01:00</t>
+          <t>2025-12-22</t>
         </is>
       </c>
     </row>

</xml_diff>